<commit_message>
Conexión excel con interfaz
</commit_message>
<xml_diff>
--- a/ProyectoSoftwareSistemas/bin/Debug/output/EJERCFINAL_ArchivoIntermedio.xlsx
+++ b/ProyectoSoftwareSistemas/bin/Debug/output/EJERCFINAL_ArchivoIntermedio.xlsx
@@ -8,6 +8,8 @@
   <x:sheets>
     <x:sheet name="ArchivoIntermedio" sheetId="1" r:id="rId2"/>
     <x:sheet name="ProgramaObjeto" sheetId="2" r:id="rId3"/>
+    <x:sheet name="TABBLK" sheetId="3" r:id="rId4"/>
+    <x:sheet name="TABSIM" sheetId="4" r:id="rId5"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="125725"/>
@@ -17,31 +19,34 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
-    <x:t>Numero de Linea</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Contador de Programa</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Etiqueta</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CodigoOp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Operador</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Formato de Instruccion</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Modo de Direccionamiento</x:t>
+    <x:t>Num. Linea</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Num. Bloque</x:t>
+  </x:si>
+  <x:si>
+    <x:t>P.C.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Etiq.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CodOp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Op</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Frmt. Inst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>M.D.</x:t>
   </x:si>
   <x:si>
     <x:t>Errores</x:t>
   </x:si>
   <x:si>
-    <x:t>Codigo Objeto</x:t>
+    <x:t>C.O.</x:t>
   </x:si>
   <x:si>
     <x:t>0000</x:t>
@@ -158,7 +163,7 @@
     <x:t>--</x:t>
   </x:si>
   <x:si>
-    <x:t>Error: Registro inválido en segundo operando</x:t>
+    <x:t>A445</x:t>
   </x:si>
   <x:si>
     <x:t>004A</x:t>
@@ -176,10 +181,10 @@
     <x:t>+LDA</x:t>
   </x:si>
   <x:si>
-    <x:t>Símbolo no encontrado</x:t>
-  </x:si>
-  <x:si>
-    <x:t>037FFFFF</x:t>
+    <x:t>Expresión vacía</x:t>
+  </x:si>
+  <x:si>
+    <x:t>033FFFFF</x:t>
   </x:si>
   <x:si>
     <x:t>004E</x:t>
@@ -239,10 +244,10 @@
     <x:t>ADD</x:t>
   </x:si>
   <x:si>
-    <x:t>Error: Operando fuera de rango</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1BEFFF</x:t>
+    <x:t>Fuera de rango</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1B3FFF</x:t>
   </x:si>
   <x:si>
     <x:t>6F5B</x:t>
@@ -251,7 +256,7 @@
     <x:t>STCH</x:t>
   </x:si>
   <x:si>
-    <x:t>566FFF</x:t>
+    <x:t>563FFF</x:t>
   </x:si>
   <x:si>
     <x:t>6F5E</x:t>
@@ -311,7 +316,7 @@
     <x:t>CADENA,X</x:t>
   </x:si>
   <x:si>
-    <x:t>Error: Símbolo no encontrado</x:t>
+    <x:t>Símbolo no definido: CADENA</x:t>
   </x:si>
   <x:si>
     <x:t>3FEFFF</x:t>
@@ -323,7 +328,7 @@
     <x:t>+TIX</x:t>
   </x:si>
   <x:si>
-    <x:t>2F7FFFFF</x:t>
+    <x:t>2F3FFFFF</x:t>
   </x:si>
   <x:si>
     <x:t>6FAF</x:t>
@@ -335,19 +340,22 @@
     <x:t>INICIO</x:t>
   </x:si>
   <x:si>
+    <x:t>Símbolo no definido: INICIO</x:t>
+  </x:si>
+  <x:si>
     <x:t>HEJERCF000000006FAF</x:t>
   </x:si>
   <x:si>
     <x:t>T00000008F00610000800008C</x:t>
   </x:si>
   <x:si>
-    <x:t>T000044126F900005037FFFFF46494E414C012FB29441</x:t>
-  </x:si>
-  <x:si>
-    <x:t>T006F58091BEFFF566FFF37AFF7</x:t>
-  </x:si>
-  <x:si>
-    <x:t>T006FA10E0F2FB41F10015E3FEFFF2F7FFFFF</x:t>
+    <x:t>T000044146F900005A445033FFFFF46494E414C012FB29441</x:t>
+  </x:si>
+  <x:si>
+    <x:t>T006F58091B3FFF563FFF37AFF7</x:t>
+  </x:si>
+  <x:si>
+    <x:t>T006FA10E0F2FB41F10015E3FEFFF2F3FFFFF</x:t>
   </x:si>
   <x:si>
     <x:t>M00000205+EJERCF</x:t>
@@ -356,7 +364,43 @@
     <x:t>M00004505+EJERCF</x:t>
   </x:si>
   <x:si>
-    <x:t>E000000</x:t>
+    <x:t>EFFFFFF</x:t>
+  </x:si>
+  <x:si>
+    <x:t>No. Bloque</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nombre</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Longitud</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Dir Inicial</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DEFAULT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Simbolo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Direccion</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Tipo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Relativo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Bloque</x:t>
+  </x:si>
+  <x:si>
+    <x:t>R</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sí</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -707,10 +751,10 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:I26"/>
+  <x:dimension ref="A1:J26"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
-    <x:row r="1" spans="1:9">
+    <x:row r="1" spans="1:10">
       <x:c r="A1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -738,13 +782,16 @@
       <x:c r="I1" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:9">
+      <x:c r="J1" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:10">
       <x:c r="A2" s="0">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>9</x:v>
+      <x:c r="B2" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
         <x:v>10</x:v>
@@ -767,48 +814,54 @@
       <x:c r="I2" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" spans="1:9">
+      <x:c r="J2" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:10">
       <x:c r="A3" s="0">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>9</x:v>
+      <x:c r="B3" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="H3" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J3" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:10">
       <x:c r="A4" s="0">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>20</x:v>
+      <x:c r="B4" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
         <x:v>22</x:v>
@@ -820,18 +873,21 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="H4" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="I4" s="0" t="s">
-        <x:v>25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J4" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:10">
       <x:c r="A5" s="0">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>26</x:v>
+      <x:c r="B5" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
         <x:v>27</x:v>
@@ -843,7 +899,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
         <x:v>14</x:v>
@@ -852,27 +908,30 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="I5" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J5" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:10">
       <x:c r="A6" s="0">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>31</x:v>
+      <x:c r="B6" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
         <x:v>33</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
         <x:v>14</x:v>
@@ -883,16 +942,19 @@
       <x:c r="I6" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" spans="1:9">
+      <x:c r="J6" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:10">
       <x:c r="A7" s="0">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>31</x:v>
+      <x:c r="B7" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
         <x:v>35</x:v>
@@ -901,7 +963,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="G7" s="0" t="s">
         <x:v>14</x:v>
@@ -912,48 +974,54 @@
       <x:c r="I7" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" spans="1:9">
+      <x:c r="J7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:10">
       <x:c r="A8" s="0">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>37</x:v>
+      <x:c r="B8" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="F8" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G8" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="H8" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="I8" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J8" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:10">
       <x:c r="A9" s="0">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>42</x:v>
+      <x:c r="B9" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
         <x:v>44</x:v>
@@ -968,114 +1036,126 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="I9" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J9" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:10">
       <x:c r="A10" s="0">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>48</x:v>
+      <x:c r="B10" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="F10" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G10" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H10" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="I10" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:9">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="J10" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:10">
       <x:c r="A11" s="0">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B11" s="0" t="s">
-        <x:v>48</x:v>
+      <x:c r="B11" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F11" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G11" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H11" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="I11" s="0" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="D11" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E11" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F11" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G11" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H11" s="0" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="I11" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" spans="1:9">
+      <x:c r="J11" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:10">
       <x:c r="A12" s="0">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B12" s="0" t="s">
-        <x:v>48</x:v>
+      <x:c r="B12" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="F12" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G12" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="H12" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="I12" s="0" t="s">
         <x:v>54</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" spans="1:9">
+      <x:c r="J12" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:10">
       <x:c r="A13" s="0">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B13" s="0" t="s">
-        <x:v>55</x:v>
+      <x:c r="B13" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="F13" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="G13" s="0" t="s">
         <x:v>14</x:v>
@@ -1084,21 +1164,24 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="I13" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" spans="1:9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J13" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:10">
       <x:c r="A14" s="0">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B14" s="0" t="s">
-        <x:v>59</x:v>
+      <x:c r="B14" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E14" s="0" t="s">
         <x:v>61</x:v>
@@ -1110,59 +1193,65 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="H14" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="I14" s="0" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" spans="1:9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J14" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:10">
       <x:c r="A15" s="0">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B15" s="0" t="s">
-        <x:v>65</x:v>
+      <x:c r="B15" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E15" s="0" t="s">
         <x:v>67</x:v>
       </x:c>
       <x:c r="F15" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="G15" s="0" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="H15" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="I15" s="0" t="s">
-        <x:v>68</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" spans="1:9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J15" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" spans="1:10">
       <x:c r="A16" s="0">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B16" s="0" t="s">
-        <x:v>69</x:v>
+      <x:c r="B16" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E16" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F16" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="G16" s="0" t="s">
         <x:v>14</x:v>
@@ -1173,13 +1262,16 @@
       <x:c r="I16" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17" spans="1:9">
+      <x:c r="J16" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:10">
       <x:c r="A17" s="0">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B17" s="0" t="s">
-        <x:v>71</x:v>
+      <x:c r="B17" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
         <x:v>72</x:v>
@@ -1188,85 +1280,94 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="E17" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="F17" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G17" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="H17" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="I17" s="0" t="s">
         <x:v>75</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" spans="1:9">
+      <x:c r="J17" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" spans="1:10">
       <x:c r="A18" s="0">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B18" s="0" t="s">
-        <x:v>76</x:v>
+      <x:c r="B18" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C18" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E18" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="F18" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G18" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="H18" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="I18" s="0" t="s">
-        <x:v>78</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" spans="1:9">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J18" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:10">
       <x:c r="A19" s="0">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B19" s="0" t="s">
-        <x:v>79</x:v>
+      <x:c r="B19" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E19" s="0" t="s">
         <x:v>81</x:v>
       </x:c>
       <x:c r="F19" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="G19" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="H19" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="I19" s="0" t="s">
-        <x:v>82</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" spans="1:9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J19" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" spans="1:10">
       <x:c r="A20" s="0">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B20" s="0" t="s">
-        <x:v>83</x:v>
+      <x:c r="B20" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
         <x:v>84</x:v>
@@ -1278,7 +1379,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="F20" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="G20" s="0" t="s">
         <x:v>14</x:v>
@@ -1289,170 +1390,188 @@
       <x:c r="I20" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21" spans="1:9">
+      <x:c r="J20" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:10">
       <x:c r="A21" s="0">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B21" s="0" t="s">
-        <x:v>87</x:v>
+      <x:c r="B21" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C21" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E21" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="F21" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="G21" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="H21" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I21" s="0" t="s">
-        <x:v>90</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" spans="1:9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J21" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" spans="1:10">
       <x:c r="A22" s="0">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B22" s="0" t="s">
-        <x:v>91</x:v>
+      <x:c r="B22" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C22" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E22" s="0" t="s">
         <x:v>93</x:v>
       </x:c>
       <x:c r="F22" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="G22" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="H22" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I22" s="0" t="s">
-        <x:v>94</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" spans="1:9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J22" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" spans="1:10">
       <x:c r="A23" s="0">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B23" s="0" t="s">
-        <x:v>95</x:v>
+      <x:c r="B23" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C23" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E23" s="0" t="s">
         <x:v>97</x:v>
       </x:c>
       <x:c r="F23" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="G23" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="H23" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="I23" s="0" t="s">
         <x:v>99</x:v>
       </x:c>
-    </x:row>
-    <x:row r="24" spans="1:9">
+      <x:c r="J23" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:10">
       <x:c r="A24" s="0">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B24" s="0" t="s">
-        <x:v>100</x:v>
+      <x:c r="B24" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C24" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E24" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="F24" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G24" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="H24" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="I24" s="0" t="s">
-        <x:v>102</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" spans="1:9">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="J24" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:10">
       <x:c r="A25" s="0">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B25" s="0" t="s">
-        <x:v>103</x:v>
+      <x:c r="B25" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C25" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E25" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="F25" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G25" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H25" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="I25" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" spans="1:9">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="J25" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:10">
       <x:c r="A26" s="0">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="B26" s="0" t="s">
-        <x:v>103</x:v>
+      <x:c r="B26" s="0">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C26" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E26" s="0" t="s">
         <x:v>105</x:v>
       </x:c>
       <x:c r="F26" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="G26" s="0" t="s">
         <x:v>14</x:v>
@@ -1461,7 +1580,10 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="I26" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="J26" s="0" t="s">
+        <x:v>17</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1481,47 +1603,223 @@
   <x:dimension ref="A1:A8"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="48.853482" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="53.282054" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:1">
       <x:c r="A1" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
       <x:c r="A2" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1">
       <x:c r="A3" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
       <x:c r="A4" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
       <x:c r="A5" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
       <x:c r="A6" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>113</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
       <x:c r="A7" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:1">
       <x:c r="A8" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>115</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:D2"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="3" width="8.853482" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8.996339" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:4">
+      <x:c r="A1" s="0" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="D1" s="0" t="s">
+        <x:v>119</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:4">
+      <x:c r="A2" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:E6"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8.282054" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="9.139196" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4.710625" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8.139196" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="8.853482" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:5">
+      <x:c r="A1" s="0" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="D1" s="0" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="E1" s="0" t="s">
+        <x:v>125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:5">
+      <x:c r="A2" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:5">
+      <x:c r="A3" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:5">
+      <x:c r="A4" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:5">
+      <x:c r="A5" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:5">
+      <x:c r="A6" s="0" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>120</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>